<commit_message>
feat: update README and add confirmation for Excel closure in the application
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran_sekolah.xlsx
+++ b/dataset/konfirm_kehadiran_sekolah.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="25600" windowHeight="12760" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="26800" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
     <col width="25.33203125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -479,75 +479,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hasan Abdum</t>
+          <t>KENZA SHAKIL AHMAD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>KENZA SHAKIL AHMAD</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Hasan Abdum</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>KENZA SHAKIL AHMAD</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-09-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Hasan Abdum</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>KENZA SHAKIL AHMAD</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-    </row>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Refactor konfirm_kehadiran.py and pendaftaran.py for improved logging and code clarity
- Removed unused imports and commented-out code in konfirm_kehadiran.py
- Simplified the register_single_entry function by removing the date_picker parameter
- Enhanced logging for various input fields in both konfirm_kehadiran.py and pendaftaran.py
- Improved error handling and user feedback during the registration process
- Updated the prepare_registration_page function to include more detailed checks for UI elements
- Cleaned up the isi_data_wali and handle_periksa_kembali functions for better readability
- Added checks for the presence of elements before interacting with them to prevent runtime errors
</commit_message>
<xml_diff>
--- a/dataset/konfirm_kehadiran_sekolah.xlsx
+++ b/dataset/konfirm_kehadiran_sekolah.xlsx
@@ -1,88 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbokprom12021/PycharmProjects/CKG-Helper/dataset/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A24C4EE-3322-5342-8F52-05A414B8A1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="26800" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="780" windowWidth="26800" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
-  <si>
-    <t>sekolah</t>
-  </si>
-  <si>
-    <t>kelas</t>
-  </si>
-  <si>
-    <t>nama_lengkap</t>
-  </si>
-  <si>
-    <t>whatsapp</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>al irsyad</t>
-  </si>
-  <si>
-    <t>Kelas 1</t>
-  </si>
-  <si>
-    <t>Ummu Salamah</t>
-  </si>
-  <si>
-    <t>8123456780</t>
-  </si>
-  <si>
-    <t>SUCCESS</t>
-  </si>
-  <si>
-    <t>Zavier Junior Hafiantono</t>
-  </si>
-  <si>
-    <t>Pasien tidak ditemukan atau sudah mengkonfirmasi kehadiran</t>
-  </si>
-  <si>
-    <t>Zain</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FF343434"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color rgb="FF343434"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -101,23 +52,82 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -437,91 +447,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16"/>
   <cols>
-    <col min="3" max="3" width="25.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.5" bestFit="1" customWidth="1"/>
+    <col width="25.33203125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" style="1" min="4" max="4"/>
+    <col width="10.5" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="11.83203125" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="14.33203125" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="10.83203125" customWidth="1" style="1" min="8" max="8"/>
+    <col width="10.83203125" customWidth="1" style="1" min="10" max="10"/>
+    <col width="16" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="13.5" bestFit="1" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sekolah</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>kelas</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>nama_lengkap</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>whatsapp</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>al irsyad</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kelas 1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Ummu Salamah</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>8123456780</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>al irsyad</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kelas 1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Zavier Junior Hafiantono</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>8123456780</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pasien tidak ditemukan atau sudah mengkonfirmasi kehadiran</t>
+        </is>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>al irsyad</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Kelas 1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Zain</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>8123456780</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>